<commit_message>
V62_DIFFSET: işaret değişimi sütunu düzeltildi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012VyUPTEQJx1C4q1PKw5aha
</commit_message>
<xml_diff>
--- a/FCF_K13/V62_DIFFSET.xlsx
+++ b/FCF_K13/V62_DIFFSET.xlsx
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,9 +64,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4790,9 +4796,7 @@
       <c r="E2" t="n">
         <v>97.09999999999999</v>
       </c>
-      <c r="F2" t="n">
-        <v/>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -4848,9 +4852,7 @@
       <c r="E3" t="n">
         <v>113.1</v>
       </c>
-      <c r="F3" t="n">
-        <v/>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -4904,11 +4906,9 @@
         <v>-509.04</v>
       </c>
       <c r="E4" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F4" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -4962,11 +4962,9 @@
         <v>-453.598</v>
       </c>
       <c r="E5" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F5" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -5020,11 +5018,9 @@
         <v>-406.026</v>
       </c>
       <c r="E6" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F6" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -5061,58 +5057,60 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>ALCAR</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>2025/03</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="2" t="n">
         <v>2259.664</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>-381.301</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="2" t="n">
         <v>-116.9</v>
       </c>
-      <c r="F7" t="n">
-        <v/>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>EVO</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>EVET</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>EVO</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>BELGE</t>
         </is>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" s="2" t="n">
         <v>-117.416</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L7" s="2" t="n">
         <v>183.997</v>
       </c>
-      <c r="M7" t="n">
+      <c r="M7" s="2" t="n">
         <v>79.88800000000001</v>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>Sistematik Evo hatası kontrolü (şirketin başka bir döneminde Evo belgeyle uyuşmadı) → Evo rakamı belgeyle uyuşmadı; belge rakamı (V7 2,259.7)</t>
         </is>
@@ -5138,9 +5136,7 @@
       <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="n">
-        <v/>
-      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -5196,9 +5192,7 @@
       <c r="E9" t="n">
         <v>0</v>
       </c>
-      <c r="F9" t="n">
-        <v/>
-      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -5254,9 +5248,7 @@
       <c r="E10" t="n">
         <v>0</v>
       </c>
-      <c r="F10" t="n">
-        <v/>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -5312,9 +5304,7 @@
       <c r="E11" t="n">
         <v>14.9</v>
       </c>
-      <c r="F11" t="n">
-        <v/>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -5370,9 +5360,7 @@
       <c r="E12" t="n">
         <v>4</v>
       </c>
-      <c r="F12" t="n">
-        <v/>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -5428,9 +5416,7 @@
       <c r="E13" t="n">
         <v>-17.8</v>
       </c>
-      <c r="F13" t="n">
-        <v/>
-      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -5486,9 +5472,7 @@
       <c r="E14" t="n">
         <v>5.9</v>
       </c>
-      <c r="F14" t="n">
-        <v/>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -5544,9 +5528,7 @@
       <c r="E15" t="n">
         <v>-1.1</v>
       </c>
-      <c r="F15" t="n">
-        <v/>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -5602,9 +5584,7 @@
       <c r="E16" t="n">
         <v>23.3</v>
       </c>
-      <c r="F16" t="n">
-        <v/>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -5660,9 +5640,7 @@
       <c r="E17" t="n">
         <v>0</v>
       </c>
-      <c r="F17" t="n">
-        <v/>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -5716,11 +5694,9 @@
         <v>2138.938</v>
       </c>
       <c r="E18" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F18" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -5776,9 +5752,7 @@
       <c r="E19" t="n">
         <v>0</v>
       </c>
-      <c r="F19" t="n">
-        <v/>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -5834,9 +5808,7 @@
       <c r="E20" t="n">
         <v>0</v>
       </c>
-      <c r="F20" t="n">
-        <v/>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -5892,9 +5864,7 @@
       <c r="E21" t="n">
         <v>0</v>
       </c>
-      <c r="F21" t="n">
-        <v/>
-      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -5950,9 +5920,7 @@
       <c r="E22" t="n">
         <v>-0.2</v>
       </c>
-      <c r="F22" t="n">
-        <v/>
-      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -6008,9 +5976,7 @@
       <c r="E23" t="n">
         <v>-3.6</v>
       </c>
-      <c r="F23" t="n">
-        <v/>
-      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -6066,9 +6032,7 @@
       <c r="E24" t="n">
         <v>-11.3</v>
       </c>
-      <c r="F24" t="n">
-        <v/>
-      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -6124,9 +6088,7 @@
       <c r="E25" t="n">
         <v>0</v>
       </c>
-      <c r="F25" t="n">
-        <v/>
-      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -6182,9 +6144,7 @@
       <c r="E26" t="n">
         <v>-31.2</v>
       </c>
-      <c r="F26" t="n">
-        <v/>
-      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -6240,9 +6200,7 @@
       <c r="E27" t="n">
         <v>0</v>
       </c>
-      <c r="F27" t="n">
-        <v/>
-      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -6296,11 +6254,9 @@
         <v>-351.894</v>
       </c>
       <c r="E28" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F28" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -6356,9 +6312,7 @@
       <c r="E29" t="n">
         <v>0</v>
       </c>
-      <c r="F29" t="n">
-        <v/>
-      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -6414,9 +6368,7 @@
       <c r="E30" t="n">
         <v>0</v>
       </c>
-      <c r="F30" t="n">
-        <v/>
-      </c>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -6472,9 +6424,7 @@
       <c r="E31" t="n">
         <v>0</v>
       </c>
-      <c r="F31" t="n">
-        <v/>
-      </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -6528,11 +6478,9 @@
         <v>-770.915</v>
       </c>
       <c r="E32" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F32" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -6588,9 +6536,7 @@
       <c r="E33" t="n">
         <v>-10.7</v>
       </c>
-      <c r="F33" t="n">
-        <v/>
-      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -6646,9 +6592,7 @@
       <c r="E34" t="n">
         <v>-15</v>
       </c>
-      <c r="F34" t="n">
-        <v/>
-      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -6704,9 +6648,7 @@
       <c r="E35" t="n">
         <v>-39.5</v>
       </c>
-      <c r="F35" t="n">
-        <v/>
-      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -6762,9 +6704,7 @@
       <c r="E36" t="n">
         <v>-2.7</v>
       </c>
-      <c r="F36" t="n">
-        <v/>
-      </c>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -6820,9 +6760,7 @@
       <c r="E37" t="n">
         <v>67.40000000000001</v>
       </c>
-      <c r="F37" t="n">
-        <v/>
-      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -6878,9 +6816,7 @@
       <c r="E38" t="n">
         <v>0</v>
       </c>
-      <c r="F38" t="n">
-        <v/>
-      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -6934,11 +6870,9 @@
         <v>972.987</v>
       </c>
       <c r="E39" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F39" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -6994,9 +6928,7 @@
       <c r="E40" t="n">
         <v>0</v>
       </c>
-      <c r="F40" t="n">
-        <v/>
-      </c>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -7050,11 +6982,9 @@
         <v>-132.54</v>
       </c>
       <c r="E41" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F41" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -7110,9 +7040,7 @@
       <c r="E42" t="n">
         <v>0</v>
       </c>
-      <c r="F42" t="n">
-        <v/>
-      </c>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -7166,11 +7094,9 @@
         <v>1847.836</v>
       </c>
       <c r="E43" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F43" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -7226,9 +7152,7 @@
       <c r="E44" t="n">
         <v>0</v>
       </c>
-      <c r="F44" t="n">
-        <v/>
-      </c>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -7284,9 +7208,7 @@
       <c r="E45" t="n">
         <v>-49.1</v>
       </c>
-      <c r="F45" t="n">
-        <v/>
-      </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -7342,9 +7264,7 @@
       <c r="E46" t="n">
         <v>-16.3</v>
       </c>
-      <c r="F46" t="n">
-        <v/>
-      </c>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -7398,11 +7318,9 @@
         <v>-784.277</v>
       </c>
       <c r="E47" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F47" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -7456,11 +7374,9 @@
         <v>-840.064</v>
       </c>
       <c r="E48" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F48" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -7516,9 +7432,7 @@
       <c r="E49" t="n">
         <v>-7.2</v>
       </c>
-      <c r="F49" t="n">
-        <v/>
-      </c>
+      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -7574,9 +7488,7 @@
       <c r="E50" t="n">
         <v>0</v>
       </c>
-      <c r="F50" t="n">
-        <v/>
-      </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -7632,9 +7544,7 @@
       <c r="E51" t="n">
         <v>0</v>
       </c>
-      <c r="F51" t="n">
-        <v/>
-      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -7690,9 +7600,7 @@
       <c r="E52" t="n">
         <v>-72.40000000000001</v>
       </c>
-      <c r="F52" t="n">
-        <v/>
-      </c>
+      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -7748,9 +7656,7 @@
       <c r="E53" t="n">
         <v>0</v>
       </c>
-      <c r="F53" t="n">
-        <v/>
-      </c>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -7806,9 +7712,7 @@
       <c r="E54" t="n">
         <v>0</v>
       </c>
-      <c r="F54" t="n">
-        <v/>
-      </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -7864,9 +7768,7 @@
       <c r="E55" t="n">
         <v>-51.5</v>
       </c>
-      <c r="F55" t="n">
-        <v/>
-      </c>
+      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -7922,9 +7824,7 @@
       <c r="E56" t="n">
         <v>0</v>
       </c>
-      <c r="F56" t="n">
-        <v/>
-      </c>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -7980,9 +7880,7 @@
       <c r="E57" t="n">
         <v>0</v>
       </c>
-      <c r="F57" t="n">
-        <v/>
-      </c>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8038,9 +7936,7 @@
       <c r="E58" t="n">
         <v>0</v>
       </c>
-      <c r="F58" t="n">
-        <v/>
-      </c>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8096,9 +7992,7 @@
       <c r="E59" t="n">
         <v>0</v>
       </c>
-      <c r="F59" t="n">
-        <v/>
-      </c>
+      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8154,9 +8048,7 @@
       <c r="E60" t="n">
         <v>0</v>
       </c>
-      <c r="F60" t="n">
-        <v/>
-      </c>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8210,11 +8102,9 @@
         <v>2038.437</v>
       </c>
       <c r="E61" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F61" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8251,116 +8141,120 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>GSDDE</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>2025/03</t>
         </is>
       </c>
-      <c r="C62" t="n">
+      <c r="C62" s="2" t="n">
         <v>-53.51800000000003</v>
       </c>
-      <c r="D62" t="n">
+      <c r="D62" s="2" t="n">
         <v>2.213</v>
       </c>
-      <c r="E62" t="n">
+      <c r="E62" s="2" t="n">
         <v>104.1</v>
       </c>
-      <c r="F62" t="n">
-        <v/>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>EVO</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>EVET</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>EVO</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
         <is>
           <t>BELGE</t>
         </is>
       </c>
-      <c r="K62" t="n">
+      <c r="K62" s="2" t="n">
         <v>410.327</v>
       </c>
-      <c r="L62" t="n">
+      <c r="L62" s="2" t="n">
         <v>404.001</v>
       </c>
-      <c r="M62" t="n">
+      <c r="M62" s="2" t="n">
         <v>4.113</v>
       </c>
-      <c r="N62" t="inlineStr">
+      <c r="N62" s="2" t="inlineStr">
         <is>
           <t>Sistematik Evo hatası kontrolü (şirketin başka bir döneminde Evo belgeyle uyuşmadı) → Evo rakamı belgeyle uyuşmadı; belge rakamı (V7 -53.5)</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>GSDDE</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>2025/06</t>
         </is>
       </c>
-      <c r="C63" t="n">
+      <c r="C63" s="2" t="n">
         <v>-11.90399999999997</v>
       </c>
-      <c r="D63" t="n">
+      <c r="D63" s="2" t="n">
         <v>43.828</v>
       </c>
-      <c r="E63" t="n">
+      <c r="E63" s="2" t="n">
         <v>468.2</v>
       </c>
-      <c r="F63" t="n">
-        <v/>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>EVO</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>EVET</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>EVO</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
         <is>
           <t>BELGE</t>
         </is>
       </c>
-      <c r="K63" t="n">
+      <c r="K63" s="2" t="n">
         <v>447.047</v>
       </c>
-      <c r="L63" t="n">
+      <c r="L63" s="2" t="n">
         <v>398.945</v>
       </c>
-      <c r="M63" t="n">
+      <c r="M63" s="2" t="n">
         <v>4.274</v>
       </c>
-      <c r="N63" t="inlineStr">
+      <c r="N63" s="2" t="inlineStr">
         <is>
           <t>Sistematik Evo hatası kontrolü (şirketin başka bir döneminde Evo belgeyle uyuşmadı) → Evo rakamı belgeyle uyuşmadı; belge rakamı (V7 -11.9)</t>
         </is>
@@ -8384,11 +8278,9 @@
         <v>151.208</v>
       </c>
       <c r="E64" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F64" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8444,9 +8336,7 @@
       <c r="E65" t="n">
         <v>-40.3</v>
       </c>
-      <c r="F65" t="n">
-        <v/>
-      </c>
+      <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8502,9 +8392,7 @@
       <c r="E66" t="n">
         <v>-18.1</v>
       </c>
-      <c r="F66" t="n">
-        <v/>
-      </c>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8560,9 +8448,7 @@
       <c r="E67" t="n">
         <v>0</v>
       </c>
-      <c r="F67" t="n">
-        <v/>
-      </c>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8618,9 +8504,7 @@
       <c r="E68" t="n">
         <v>0</v>
       </c>
-      <c r="F68" t="n">
-        <v/>
-      </c>
+      <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8676,9 +8560,7 @@
       <c r="E69" t="n">
         <v>0</v>
       </c>
-      <c r="F69" t="n">
-        <v/>
-      </c>
+      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -8734,9 +8616,7 @@
       <c r="E70" t="n">
         <v>36.7</v>
       </c>
-      <c r="F70" t="n">
-        <v/>
-      </c>
+      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8792,9 +8672,7 @@
       <c r="E71" t="n">
         <v>33.3</v>
       </c>
-      <c r="F71" t="n">
-        <v/>
-      </c>
+      <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8848,11 +8726,9 @@
         <v>-858.465</v>
       </c>
       <c r="E72" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F72" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8906,11 +8782,9 @@
         <v>-438.889</v>
       </c>
       <c r="E73" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F73" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -8966,9 +8840,7 @@
       <c r="E74" t="n">
         <v>0</v>
       </c>
-      <c r="F74" t="n">
-        <v/>
-      </c>
+      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9024,9 +8896,7 @@
       <c r="E75" t="n">
         <v>-7335.3</v>
       </c>
-      <c r="F75" t="n">
-        <v/>
-      </c>
+      <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9080,11 +8950,9 @@
         <v>-652.2380000000001</v>
       </c>
       <c r="E76" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F76" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9138,11 +9006,9 @@
         <v>-657.917</v>
       </c>
       <c r="E77" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F77" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9196,11 +9062,9 @@
         <v>-771.954</v>
       </c>
       <c r="E78" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F78" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9256,9 +9120,7 @@
       <c r="E79" t="n">
         <v>76.2</v>
       </c>
-      <c r="F79" t="n">
-        <v/>
-      </c>
+      <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9314,9 +9176,7 @@
       <c r="E80" t="n">
         <v>6.7</v>
       </c>
-      <c r="F80" t="n">
-        <v/>
-      </c>
+      <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9372,9 +9232,7 @@
       <c r="E81" t="n">
         <v>-35.5</v>
       </c>
-      <c r="F81" t="n">
-        <v/>
-      </c>
+      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9430,9 +9288,7 @@
       <c r="E82" t="n">
         <v>-62.6</v>
       </c>
-      <c r="F82" t="n">
-        <v/>
-      </c>
+      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9488,9 +9344,7 @@
       <c r="E83" t="n">
         <v>0</v>
       </c>
-      <c r="F83" t="n">
-        <v/>
-      </c>
+      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9546,9 +9400,7 @@
       <c r="E84" t="n">
         <v>0</v>
       </c>
-      <c r="F84" t="n">
-        <v/>
-      </c>
+      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9604,9 +9456,7 @@
       <c r="E85" t="n">
         <v>0</v>
       </c>
-      <c r="F85" t="n">
-        <v/>
-      </c>
+      <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9643,58 +9493,60 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>IZMDC</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr">
         <is>
           <t>2025/06</t>
         </is>
       </c>
-      <c r="C86" t="n">
+      <c r="C86" s="2" t="n">
         <v>121.025999999999</v>
       </c>
-      <c r="D86" t="n">
+      <c r="D86" s="2" t="n">
         <v>-2021.3</v>
       </c>
-      <c r="E86" t="n">
+      <c r="E86" s="2" t="n">
         <v>-1770.1</v>
       </c>
-      <c r="F86" t="n">
-        <v/>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>EVO</t>
-        </is>
-      </c>
-      <c r="J86" t="inlineStr">
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>EVET</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>EVO</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
         <is>
           <t>BELGE</t>
         </is>
       </c>
-      <c r="K86" t="n">
+      <c r="K86" s="2" t="n">
         <v>843.078</v>
       </c>
-      <c r="L86" t="n">
+      <c r="L86" s="2" t="n">
         <v>2782.783</v>
       </c>
-      <c r="M86" t="n">
+      <c r="M86" s="2" t="n">
         <v>81.595</v>
       </c>
-      <c r="N86" t="inlineStr">
+      <c r="N86" s="2" t="inlineStr">
         <is>
           <t>Sistematik Evo hatası kontrolü (şirketin başka bir döneminde Evo belgeyle uyuşmadı) → Evo rakamı belgeyle uyuşmadı; belge rakamı (V7 121.0)</t>
         </is>
@@ -9720,9 +9572,7 @@
       <c r="E87" t="n">
         <v>0</v>
       </c>
-      <c r="F87" t="n">
-        <v/>
-      </c>
+      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9778,9 +9628,7 @@
       <c r="E88" t="n">
         <v>0</v>
       </c>
-      <c r="F88" t="n">
-        <v/>
-      </c>
+      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9836,9 +9684,7 @@
       <c r="E89" t="n">
         <v>0</v>
       </c>
-      <c r="F89" t="n">
-        <v/>
-      </c>
+      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -9892,11 +9738,9 @@
         <v>-1648.407</v>
       </c>
       <c r="E90" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F90" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -9950,11 +9794,9 @@
         <v>-767.428</v>
       </c>
       <c r="E91" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F91" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -10008,11 +9850,9 @@
         <v>-1407.557</v>
       </c>
       <c r="E92" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F92" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -10066,11 +9906,9 @@
         <v>934.352</v>
       </c>
       <c r="E93" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F93" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -10126,9 +9964,7 @@
       <c r="E94" t="n">
         <v>0</v>
       </c>
-      <c r="F94" t="n">
-        <v/>
-      </c>
+      <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -10182,11 +10018,9 @@
         <v>-2807.813</v>
       </c>
       <c r="E95" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F95" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -10240,11 +10074,9 @@
         <v>-2807.813</v>
       </c>
       <c r="E96" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F96" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -10298,11 +10130,9 @@
         <v>-2807.813</v>
       </c>
       <c r="E97" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F97" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -10358,9 +10188,7 @@
       <c r="E98" t="n">
         <v>0</v>
       </c>
-      <c r="F98" t="n">
-        <v/>
-      </c>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -10414,11 +10242,9 @@
         <v>246.838</v>
       </c>
       <c r="E99" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F99" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -10472,11 +10298,9 @@
         <v>-609.551</v>
       </c>
       <c r="E100" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F100" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -10513,58 +10337,60 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
+      <c r="A101" s="2" t="inlineStr">
         <is>
           <t>KUVVA</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B101" s="2" t="inlineStr">
         <is>
           <t>2025/06</t>
         </is>
       </c>
-      <c r="C101" t="n">
+      <c r="C101" s="2" t="n">
         <v>-5.794999999999959</v>
       </c>
-      <c r="D101" t="n">
+      <c r="D101" s="2" t="n">
         <v>1041.809</v>
       </c>
-      <c r="E101" t="n">
+      <c r="E101" s="2" t="n">
         <v>18077.7</v>
       </c>
-      <c r="F101" t="n">
-        <v/>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="H101" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>EVO</t>
-        </is>
-      </c>
-      <c r="J101" t="inlineStr">
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>EVET</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>EVO</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
         <is>
           <t>BELGE</t>
         </is>
       </c>
-      <c r="K101" t="n">
+      <c r="K101" s="2" t="n">
         <v>2376.27</v>
       </c>
-      <c r="L101" t="n">
+      <c r="L101" s="2" t="n">
         <v>1334.461</v>
       </c>
-      <c r="M101" t="n">
-        <v>0</v>
-      </c>
-      <c r="N101" t="inlineStr">
+      <c r="M101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N101" s="2" t="inlineStr">
         <is>
           <t>Sistematik Evo hatası kontrolü (şirketin başka bir döneminde Evo belgeyle uyuşmadı) → Evo rakamı belgeyle uyuşmadı; belge rakamı (V7 -5.8)</t>
         </is>
@@ -10590,9 +10416,7 @@
       <c r="E102" t="n">
         <v>0</v>
       </c>
-      <c r="F102" t="n">
-        <v/>
-      </c>
+      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -10648,9 +10472,7 @@
       <c r="E103" t="n">
         <v>-1.9</v>
       </c>
-      <c r="F103" t="n">
-        <v/>
-      </c>
+      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -10706,9 +10528,7 @@
       <c r="E104" t="n">
         <v>0</v>
       </c>
-      <c r="F104" t="n">
-        <v/>
-      </c>
+      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -10764,9 +10584,7 @@
       <c r="E105" t="n">
         <v>0</v>
       </c>
-      <c r="F105" t="n">
-        <v/>
-      </c>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -10822,9 +10640,7 @@
       <c r="E106" t="n">
         <v>0</v>
       </c>
-      <c r="F106" t="n">
-        <v/>
-      </c>
+      <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -10880,9 +10696,7 @@
       <c r="E107" t="n">
         <v>6</v>
       </c>
-      <c r="F107" t="n">
-        <v/>
-      </c>
+      <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -10938,9 +10752,7 @@
       <c r="E108" t="n">
         <v>3.1</v>
       </c>
-      <c r="F108" t="n">
-        <v/>
-      </c>
+      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -10994,11 +10806,9 @@
         <v>-615.0700000000001</v>
       </c>
       <c r="E109" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F109" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11054,9 +10864,7 @@
       <c r="E110" t="n">
         <v>0</v>
       </c>
-      <c r="F110" t="n">
-        <v/>
-      </c>
+      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11110,11 +10918,9 @@
         <v>-2105.046</v>
       </c>
       <c r="E111" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F111" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11170,9 +10976,7 @@
       <c r="E112" t="n">
         <v>-32.3</v>
       </c>
-      <c r="F112" t="n">
-        <v/>
-      </c>
+      <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11228,9 +11032,7 @@
       <c r="E113" t="n">
         <v>-62.9</v>
       </c>
-      <c r="F113" t="n">
-        <v/>
-      </c>
+      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11286,9 +11088,7 @@
       <c r="E114" t="n">
         <v>-52.3</v>
       </c>
-      <c r="F114" t="n">
-        <v/>
-      </c>
+      <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11344,9 +11144,7 @@
       <c r="E115" t="n">
         <v>-64.7</v>
       </c>
-      <c r="F115" t="n">
-        <v/>
-      </c>
+      <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11402,9 +11200,7 @@
       <c r="E116" t="n">
         <v>-17.8</v>
       </c>
-      <c r="F116" t="n">
-        <v/>
-      </c>
+      <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11460,9 +11256,7 @@
       <c r="E117" t="n">
         <v>0</v>
       </c>
-      <c r="F117" t="n">
-        <v/>
-      </c>
+      <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -11518,9 +11312,7 @@
       <c r="E118" t="n">
         <v>0</v>
       </c>
-      <c r="F118" t="n">
-        <v/>
-      </c>
+      <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -11574,11 +11366,9 @@
         <v>244.415</v>
       </c>
       <c r="E119" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F119" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11634,9 +11424,7 @@
       <c r="E120" t="n">
         <v>0</v>
       </c>
-      <c r="F120" t="n">
-        <v/>
-      </c>
+      <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11690,11 +11478,9 @@
         <v>-1015.452</v>
       </c>
       <c r="E121" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F121" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11750,9 +11536,7 @@
       <c r="E122" t="n">
         <v>-2.5</v>
       </c>
-      <c r="F122" t="n">
-        <v/>
-      </c>
+      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11808,9 +11592,7 @@
       <c r="E123" t="n">
         <v>-8</v>
       </c>
-      <c r="F123" t="n">
-        <v/>
-      </c>
+      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11866,9 +11648,7 @@
       <c r="E124" t="n">
         <v>24.6</v>
       </c>
-      <c r="F124" t="n">
-        <v/>
-      </c>
+      <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11924,9 +11704,7 @@
       <c r="E125" t="n">
         <v>12.8</v>
       </c>
-      <c r="F125" t="n">
-        <v/>
-      </c>
+      <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -11982,9 +11760,7 @@
       <c r="E126" t="n">
         <v>0</v>
       </c>
-      <c r="F126" t="n">
-        <v/>
-      </c>
+      <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12040,9 +11816,7 @@
       <c r="E127" t="n">
         <v>0</v>
       </c>
-      <c r="F127" t="n">
-        <v/>
-      </c>
+      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12098,9 +11872,7 @@
       <c r="E128" t="n">
         <v>-64.7</v>
       </c>
-      <c r="F128" t="n">
-        <v/>
-      </c>
+      <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12156,9 +11928,7 @@
       <c r="E129" t="n">
         <v>-36.7</v>
       </c>
-      <c r="F129" t="n">
-        <v/>
-      </c>
+      <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12214,9 +11984,7 @@
       <c r="E130" t="n">
         <v>0</v>
       </c>
-      <c r="F130" t="n">
-        <v/>
-      </c>
+      <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12270,11 +12038,9 @@
         <v>225.589</v>
       </c>
       <c r="E131" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F131" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12328,11 +12094,9 @@
         <v>200.311</v>
       </c>
       <c r="E132" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F132" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12388,9 +12152,7 @@
       <c r="E133" t="n">
         <v>0</v>
       </c>
-      <c r="F133" t="n">
-        <v/>
-      </c>
+      <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12446,9 +12208,7 @@
       <c r="E134" t="n">
         <v>0</v>
       </c>
-      <c r="F134" t="n">
-        <v/>
-      </c>
+      <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12504,9 +12264,7 @@
       <c r="E135" t="n">
         <v>0</v>
       </c>
-      <c r="F135" t="n">
-        <v/>
-      </c>
+      <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12562,9 +12320,7 @@
       <c r="E136" t="n">
         <v>0</v>
       </c>
-      <c r="F136" t="n">
-        <v/>
-      </c>
+      <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12620,9 +12376,7 @@
       <c r="E137" t="n">
         <v>0</v>
       </c>
-      <c r="F137" t="n">
-        <v/>
-      </c>
+      <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12676,11 +12430,9 @@
         <v>188.421</v>
       </c>
       <c r="E138" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F138" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12734,11 +12486,9 @@
         <v>9.602</v>
       </c>
       <c r="E139" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F139" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12794,9 +12544,7 @@
       <c r="E140" t="n">
         <v>14.6</v>
       </c>
-      <c r="F140" t="n">
-        <v/>
-      </c>
+      <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12852,9 +12600,7 @@
       <c r="E141" t="n">
         <v>52.3</v>
       </c>
-      <c r="F141" t="n">
-        <v/>
-      </c>
+      <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12908,11 +12654,9 @@
         <v>-649.955</v>
       </c>
       <c r="E142" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F142" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -12966,11 +12710,9 @@
         <v>156.391</v>
       </c>
       <c r="E143" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F143" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13024,11 +12766,9 @@
         <v>169.908</v>
       </c>
       <c r="E144" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F144" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13084,9 +12824,7 @@
       <c r="E145" t="n">
         <v>-8.4</v>
       </c>
-      <c r="F145" t="n">
-        <v/>
-      </c>
+      <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13142,9 +12880,7 @@
       <c r="E146" t="n">
         <v>-9.4</v>
       </c>
-      <c r="F146" t="n">
-        <v/>
-      </c>
+      <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13200,9 +12936,7 @@
       <c r="E147" t="n">
         <v>-0.3</v>
       </c>
-      <c r="F147" t="n">
-        <v/>
-      </c>
+      <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13258,9 +12992,7 @@
       <c r="E148" t="n">
         <v>-1</v>
       </c>
-      <c r="F148" t="n">
-        <v/>
-      </c>
+      <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13316,9 +13048,7 @@
       <c r="E149" t="n">
         <v>17.1</v>
       </c>
-      <c r="F149" t="n">
-        <v/>
-      </c>
+      <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13374,9 +13104,7 @@
       <c r="E150" t="n">
         <v>367.7</v>
       </c>
-      <c r="F150" t="n">
-        <v/>
-      </c>
+      <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -13432,9 +13160,7 @@
       <c r="E151" t="n">
         <v>0</v>
       </c>
-      <c r="F151" t="n">
-        <v/>
-      </c>
+      <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13490,9 +13216,7 @@
       <c r="E152" t="n">
         <v>0</v>
       </c>
-      <c r="F152" t="n">
-        <v/>
-      </c>
+      <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13548,9 +13272,7 @@
       <c r="E153" t="n">
         <v>0</v>
       </c>
-      <c r="F153" t="n">
-        <v/>
-      </c>
+      <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13587,116 +13309,120 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr">
+      <c r="A154" s="2" t="inlineStr">
         <is>
           <t>SMART</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
+      <c r="B154" s="2" t="inlineStr">
         <is>
           <t>2025/03</t>
         </is>
       </c>
-      <c r="C154" t="n">
+      <c r="C154" s="2" t="n">
         <v>9.475000000000012</v>
       </c>
-      <c r="D154" t="n">
+      <c r="D154" s="2" t="n">
         <v>-47.207</v>
       </c>
-      <c r="E154" t="n">
+      <c r="E154" s="2" t="n">
         <v>-598.2</v>
       </c>
-      <c r="F154" t="n">
-        <v/>
-      </c>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="H154" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="I154" t="inlineStr">
-        <is>
-          <t>EVO</t>
-        </is>
-      </c>
-      <c r="J154" t="inlineStr">
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>EVET</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>EVO</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr">
         <is>
           <t>BELGE</t>
         </is>
       </c>
-      <c r="K154" t="n">
+      <c r="K154" s="2" t="n">
         <v>168.467</v>
       </c>
-      <c r="L154" t="n">
+      <c r="L154" s="2" t="n">
         <v>214.154</v>
       </c>
-      <c r="M154" t="n">
+      <c r="M154" s="2" t="n">
         <v>1.52</v>
       </c>
-      <c r="N154" t="inlineStr">
+      <c r="N154" s="2" t="inlineStr">
         <is>
           <t>Sistematik Evo hatası kontrolü (şirketin başka bir döneminde Evo belgeyle uyuşmadı) → Evo rakamı belgeyle uyuşmadı; belge rakamı (V7 9.5)</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="inlineStr">
+      <c r="A155" s="2" t="inlineStr">
         <is>
           <t>SMART</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
+      <c r="B155" s="2" t="inlineStr">
         <is>
           <t>2025/06</t>
         </is>
       </c>
-      <c r="C155" t="n">
+      <c r="C155" s="2" t="n">
         <v>7.325000000000009</v>
       </c>
-      <c r="D155" t="n">
+      <c r="D155" s="2" t="n">
         <v>-49.358</v>
       </c>
-      <c r="E155" t="n">
+      <c r="E155" s="2" t="n">
         <v>-773.8</v>
       </c>
-      <c r="F155" t="n">
-        <v/>
-      </c>
-      <c r="G155" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="H155" t="inlineStr">
-        <is>
-          <t>KESİN</t>
-        </is>
-      </c>
-      <c r="I155" t="inlineStr">
-        <is>
-          <t>EVO</t>
-        </is>
-      </c>
-      <c r="J155" t="inlineStr">
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>EVET</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>KESİN</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="inlineStr">
+        <is>
+          <t>EVO</t>
+        </is>
+      </c>
+      <c r="J155" s="2" t="inlineStr">
         <is>
           <t>BELGE</t>
         </is>
       </c>
-      <c r="K155" t="n">
+      <c r="K155" s="2" t="n">
         <v>151.335</v>
       </c>
-      <c r="L155" t="n">
+      <c r="L155" s="2" t="n">
         <v>199</v>
       </c>
-      <c r="M155" t="n">
+      <c r="M155" s="2" t="n">
         <v>1.693</v>
       </c>
-      <c r="N155" t="inlineStr">
+      <c r="N155" s="2" t="inlineStr">
         <is>
           <t>Sistematik Evo hatası kontrolü (şirketin başka bir döneminde Evo belgeyle uyuşmadı) → Evo rakamı belgeyle uyuşmadı; belge rakamı (V7 7.3)</t>
         </is>
@@ -13722,9 +13448,7 @@
       <c r="E156" t="n">
         <v>0</v>
       </c>
-      <c r="F156" t="n">
-        <v/>
-      </c>
+      <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13780,9 +13504,7 @@
       <c r="E157" t="n">
         <v>0.1</v>
       </c>
-      <c r="F157" t="n">
-        <v/>
-      </c>
+      <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13838,9 +13560,7 @@
       <c r="E158" t="n">
         <v>0.1</v>
       </c>
-      <c r="F158" t="n">
-        <v/>
-      </c>
+      <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13896,9 +13616,7 @@
       <c r="E159" t="n">
         <v>-27.9</v>
       </c>
-      <c r="F159" t="n">
-        <v/>
-      </c>
+      <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -13954,9 +13672,7 @@
       <c r="E160" t="n">
         <v>-49.6</v>
       </c>
-      <c r="F160" t="n">
-        <v/>
-      </c>
+      <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14012,9 +13728,7 @@
       <c r="E161" t="n">
         <v>-6.6</v>
       </c>
-      <c r="F161" t="n">
-        <v/>
-      </c>
+      <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14070,9 +13784,7 @@
       <c r="E162" t="n">
         <v>-7.5</v>
       </c>
-      <c r="F162" t="n">
-        <v/>
-      </c>
+      <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14128,9 +13840,7 @@
       <c r="E163" t="n">
         <v>-1.2</v>
       </c>
-      <c r="F163" t="n">
-        <v/>
-      </c>
+      <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14184,11 +13894,9 @@
         <v>275.087</v>
       </c>
       <c r="E164" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F164" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14242,11 +13950,9 @@
         <v>554.2569999999999</v>
       </c>
       <c r="E165" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F165" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14302,9 +14008,7 @@
       <c r="E166" t="n">
         <v>-65</v>
       </c>
-      <c r="F166" t="n">
-        <v/>
-      </c>
+      <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14360,9 +14064,7 @@
       <c r="E167" t="n">
         <v>0</v>
       </c>
-      <c r="F167" t="n">
-        <v/>
-      </c>
+      <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14418,9 +14120,7 @@
       <c r="E168" t="n">
         <v>0</v>
       </c>
-      <c r="F168" t="n">
-        <v/>
-      </c>
+      <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14476,9 +14176,7 @@
       <c r="E169" t="n">
         <v>0</v>
       </c>
-      <c r="F169" t="n">
-        <v/>
-      </c>
+      <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14534,9 +14232,7 @@
       <c r="E170" t="n">
         <v>0</v>
       </c>
-      <c r="F170" t="n">
-        <v/>
-      </c>
+      <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14592,9 +14288,7 @@
       <c r="E171" t="n">
         <v>4</v>
       </c>
-      <c r="F171" t="n">
-        <v/>
-      </c>
+      <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -14650,9 +14344,7 @@
       <c r="E172" t="n">
         <v>-54.6</v>
       </c>
-      <c r="F172" t="n">
-        <v/>
-      </c>
+      <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -14708,9 +14400,7 @@
       <c r="E173" t="n">
         <v>-1.3</v>
       </c>
-      <c r="F173" t="n">
-        <v/>
-      </c>
+      <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14766,9 +14456,7 @@
       <c r="E174" t="n">
         <v>-0.4</v>
       </c>
-      <c r="F174" t="n">
-        <v/>
-      </c>
+      <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -14824,9 +14512,7 @@
       <c r="E175" t="n">
         <v>0</v>
       </c>
-      <c r="F175" t="n">
-        <v/>
-      </c>
+      <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14880,11 +14566,9 @@
         <v>5914.446</v>
       </c>
       <c r="E176" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F176" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14940,9 +14624,7 @@
       <c r="E177" t="n">
         <v>0</v>
       </c>
-      <c r="F177" t="n">
-        <v/>
-      </c>
+      <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -14998,9 +14680,7 @@
       <c r="E178" t="n">
         <v>22.1</v>
       </c>
-      <c r="F178" t="n">
-        <v/>
-      </c>
+      <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15056,9 +14736,7 @@
       <c r="E179" t="n">
         <v>0</v>
       </c>
-      <c r="F179" t="n">
-        <v/>
-      </c>
+      <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15112,11 +14790,9 @@
         <v>3682.719</v>
       </c>
       <c r="E180" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F180" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15172,9 +14848,7 @@
       <c r="E181" t="n">
         <v>0</v>
       </c>
-      <c r="F181" t="n">
-        <v/>
-      </c>
+      <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15230,9 +14904,7 @@
       <c r="E182" t="n">
         <v>-10</v>
       </c>
-      <c r="F182" t="n">
-        <v/>
-      </c>
+      <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
           <t>TÜRETİLMİŞ</t>
@@ -15288,9 +14960,7 @@
       <c r="E183" t="n">
         <v>22.2</v>
       </c>
-      <c r="F183" t="n">
-        <v/>
-      </c>
+      <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15344,11 +15014,9 @@
         <v>-1157.812</v>
       </c>
       <c r="E184" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F184" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15404,9 +15072,7 @@
       <c r="E185" t="n">
         <v>-1.1</v>
       </c>
-      <c r="F185" t="n">
-        <v/>
-      </c>
+      <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15460,11 +15126,9 @@
         <v>-2456.823</v>
       </c>
       <c r="E186" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F186" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15520,9 +15184,7 @@
       <c r="E187" t="n">
         <v>0</v>
       </c>
-      <c r="F187" t="n">
-        <v/>
-      </c>
+      <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15578,9 +15240,7 @@
       <c r="E188" t="n">
         <v>0</v>
       </c>
-      <c r="F188" t="n">
-        <v/>
-      </c>
+      <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15627,14 +15287,10 @@
           <t>2025/06</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr"/>
       <c r="D189" t="n">
         <v>-0.887</v>
       </c>
-      <c r="E189" t="inlineStr"/>
-      <c r="F189" t="n">
-        <v/>
-      </c>
+      <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
           <t>NULL</t>
@@ -15690,9 +15346,7 @@
       <c r="E190" t="n">
         <v>-22.6</v>
       </c>
-      <c r="F190" t="n">
-        <v/>
-      </c>
+      <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15748,9 +15402,7 @@
       <c r="E191" t="n">
         <v>7</v>
       </c>
-      <c r="F191" t="n">
-        <v/>
-      </c>
+      <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15804,11 +15456,9 @@
         <v>-435.993</v>
       </c>
       <c r="E192" t="n">
-        <v>-0</v>
-      </c>
-      <c r="F192" t="n">
-        <v/>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15864,9 +15514,7 @@
       <c r="E193" t="n">
         <v>0</v>
       </c>
-      <c r="F193" t="n">
-        <v/>
-      </c>
+      <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
           <t>KESİN</t>
@@ -15922,9 +15570,7 @@
       <c r="E194" t="n">
         <v>0</v>
       </c>
-      <c r="F194" t="n">
-        <v/>
-      </c>
+      <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
           <t>KESİN</t>

</xml_diff>